<commit_message>
actualización proyectos, noticias y ppt
</commit_message>
<xml_diff>
--- a/data/biblioteca.xlsx
+++ b/data/biblioteca.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7bd4bafa3350f995/04. Trabajos/0. Equidad Urbana Consultora/0. EU RESPALDO 2020-2025/03.  Estudios/equidad-comunidades/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_4BBD797934D97D8E43CB55DCD104598F85806C24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77C583B6-079B-4098-9817-31AA4A63B74B}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_4BBD797934D97D8E43CB55DCD104598F85806C24" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0C4EBE2-9D08-4FFC-ADD9-543062B0FAC4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -97,30 +97,9 @@
     <t>Presentación utilizada en el taller de Uso, cuidado y mantención de las viviendas y el espacio público.</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/1YqGQ0yNbTodJMwrgY1aXVX5JJOWBalSm/view?usp=drive_link</t>
-  </si>
-  <si>
     <t>Taller de DYD</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/1UCoG2GkLQ80JmxE3BUZxuROdh3ZK0qp0/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>Taller de Redes Comunitarias</t>
-  </si>
-  <si>
-    <t>Presentación utilizada en el taller de Redes Comunitarias.</t>
-  </si>
-  <si>
-    <t>Taller de Organización Comunitaria</t>
-  </si>
-  <si>
-    <t>Presentación utilizada en el taller de Organización comunitaria.</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1YeMOaN1-ETZgMXaoVehEBIpdTm7cjhTV/view?usp=drive_link</t>
-  </si>
-  <si>
     <t>Decreto Supremo 19</t>
   </si>
   <si>
@@ -239,6 +218,12 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1ijeneq1fh6blcDjE1NSUIx2etCqg5llv/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/13RxyPJi0v0Q-nnpHGj2GGRzZfq-ya-9a/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1XcpXMmKlYudz1hGNveXlDiqYKhXtQPX7/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -277,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -288,6 +273,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="54.5703125" customWidth="1"/>
@@ -531,13 +517,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>5</v>
@@ -565,13 +551,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -599,13 +585,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>14</v>
@@ -616,13 +602,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
@@ -656,7 +642,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -676,7 +662,7 @@
         <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -684,33 +670,36 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -718,7 +707,7 @@
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>31</v>
@@ -729,155 +718,121 @@
     </row>
     <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>33</v>
       </c>
       <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" t="s">
         <v>35</v>
       </c>
-      <c r="E14" t="s">
+    </row>
+    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+    <row r="16" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" t="s">
         <v>37</v>
       </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="B18" t="s">
         <v>57</v>
       </c>
-      <c r="E17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>18</v>
-      </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" t="s">
         <v>59</v>
-      </c>
-      <c r="E18" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>60</v>
       </c>
       <c r="C19" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>62</v>
       </c>
-      <c r="E19" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>20</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C20" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>65</v>
-      </c>
-      <c r="E20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>21</v>
-      </c>
-      <c r="B21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>22</v>
-      </c>
-      <c r="B22" t="s">
-        <v>70</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>